<commit_message>
Problem: min. cost to cut a stick
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82DD34B4-B6E4-4EA2-8044-790E58BC9660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13F8EBB-27CC-4BF3-B711-94505BA59404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="550">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="552">
   <si>
     <t>date</t>
   </si>
@@ -1670,6 +1670,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/house-robber-iii/</t>
+  </si>
+  <si>
+    <t>minimum cost to cut a stick</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-cost-to-cut-a-stick/</t>
   </si>
 </sst>
 </file>
@@ -1940,7 +1946,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D275"/>
+  <dimension ref="A1:D276"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4964,6 +4970,17 @@
       </c>
       <c r="C275" s="4" t="s">
         <v>549</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A276" s="1">
+        <v>45885</v>
+      </c>
+      <c r="B276" t="s">
+        <v>550</v>
+      </c>
+      <c r="C276" s="4" t="s">
+        <v>551</v>
       </c>
     </row>
   </sheetData>
@@ -5236,8 +5253,9 @@
     <hyperlink ref="C273" r:id="rId266" xr:uid="{6C8F2F70-18CC-4A18-B5CA-CF7E77991D2E}"/>
     <hyperlink ref="C274" r:id="rId267" xr:uid="{038291A3-04CE-408E-BB32-9B5BBA6F8905}"/>
     <hyperlink ref="C275" r:id="rId268" xr:uid="{0A48FAD0-52AB-43DD-8262-D4E05CD2BB31}"/>
+    <hyperlink ref="C276" r:id="rId269" xr:uid="{729C6CA3-C94D-48A4-BEDB-9A63C93E84E8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId269"/>
+  <pageSetup orientation="portrait" r:id="rId270"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: Number of Provinces
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13F8EBB-27CC-4BF3-B711-94505BA59404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D3B856-28F8-474E-BA2B-A6F9AEF5D521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="554">
   <si>
     <t>date</t>
   </si>
@@ -1676,6 +1676,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-cost-to-cut-a-stick/</t>
+  </si>
+  <si>
+    <t>Number of provinces</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/number-of-provinces/</t>
   </si>
 </sst>
 </file>
@@ -1946,7 +1952,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D276"/>
+  <dimension ref="A1:D277"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4974,13 +4980,24 @@
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A276" s="1">
-        <v>45885</v>
+        <v>46250</v>
       </c>
       <c r="B276" t="s">
         <v>550</v>
       </c>
       <c r="C276" s="4" t="s">
         <v>551</v>
+      </c>
+    </row>
+    <row r="277" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A277" s="1">
+        <v>46254</v>
+      </c>
+      <c r="B277" t="s">
+        <v>552</v>
+      </c>
+      <c r="C277" s="4" t="s">
+        <v>553</v>
       </c>
     </row>
   </sheetData>
@@ -5254,8 +5271,9 @@
     <hyperlink ref="C274" r:id="rId267" xr:uid="{038291A3-04CE-408E-BB32-9B5BBA6F8905}"/>
     <hyperlink ref="C275" r:id="rId268" xr:uid="{0A48FAD0-52AB-43DD-8262-D4E05CD2BB31}"/>
     <hyperlink ref="C276" r:id="rId269" xr:uid="{729C6CA3-C94D-48A4-BEDB-9A63C93E84E8}"/>
+    <hyperlink ref="C277" r:id="rId270" xr:uid="{C1C5C25D-3E9A-4E13-A1BB-54B6CFF8BC72}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId270"/>
+  <pageSetup orientation="portrait" r:id="rId271"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem : Flood Fill
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F0EAC0-5692-4305-BB4C-3A71387422FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{278721D5-8E93-41A8-A326-C979180E1560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="558">
   <si>
     <t>date</t>
   </si>
@@ -1688,6 +1688,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/rotting-oranges/</t>
+  </si>
+  <si>
+    <t>Flood Fill</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/flood-fill/</t>
   </si>
 </sst>
 </file>
@@ -1958,7 +1964,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D278"/>
+  <dimension ref="A1:D279"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5015,6 +5021,17 @@
       </c>
       <c r="C278" s="4" t="s">
         <v>555</v>
+      </c>
+    </row>
+    <row r="279" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A279" s="1">
+        <v>46258</v>
+      </c>
+      <c r="B279" t="s">
+        <v>556</v>
+      </c>
+      <c r="C279" s="4" t="s">
+        <v>557</v>
       </c>
     </row>
   </sheetData>
@@ -5290,8 +5307,9 @@
     <hyperlink ref="C276" r:id="rId269" xr:uid="{729C6CA3-C94D-48A4-BEDB-9A63C93E84E8}"/>
     <hyperlink ref="C277" r:id="rId270" xr:uid="{C1C5C25D-3E9A-4E13-A1BB-54B6CFF8BC72}"/>
     <hyperlink ref="C278" r:id="rId271" xr:uid="{ADC0E283-5290-4A7E-B031-1E33BB5B8047}"/>
+    <hyperlink ref="C279" r:id="rId272" xr:uid="{EE8670A5-7218-415D-ACAC-75BB144ABB37}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId272"/>
+  <pageSetup orientation="portrait" r:id="rId273"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: No. of Enclaves
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F028FC1-756C-4E6C-A13B-276404BC91CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0959C264-A5EE-4EC4-BF27-012CF1A4F36E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="562">
   <si>
     <t>date</t>
   </si>
@@ -1700,6 +1700,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/01-matrix/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/number-of-enclaves/</t>
+  </si>
+  <si>
+    <t>No. of enclaves</t>
   </si>
 </sst>
 </file>
@@ -1970,7 +1976,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D280"/>
+  <dimension ref="A1:D281"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5049,6 +5055,17 @@
       </c>
       <c r="C280" s="4" t="s">
         <v>559</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A281" s="1">
+        <v>46259</v>
+      </c>
+      <c r="B281" t="s">
+        <v>561</v>
+      </c>
+      <c r="C281" s="4" t="s">
+        <v>560</v>
       </c>
     </row>
   </sheetData>
@@ -5326,8 +5343,9 @@
     <hyperlink ref="C278" r:id="rId271" xr:uid="{ADC0E283-5290-4A7E-B031-1E33BB5B8047}"/>
     <hyperlink ref="C279" r:id="rId272" xr:uid="{EE8670A5-7218-415D-ACAC-75BB144ABB37}"/>
     <hyperlink ref="C280" r:id="rId273" xr:uid="{CF717DFE-6659-495F-BFC7-5075CE2DA2EB}"/>
+    <hyperlink ref="C281" r:id="rId274" xr:uid="{3AC2CD71-6543-4022-99C0-EC7F6F7C2CDE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId274"/>
+  <pageSetup orientation="portrait" r:id="rId275"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: Word Ladder II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0959C264-A5EE-4EC4-BF27-012CF1A4F36E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBC68A62-C8B3-4B7C-8302-13300FA9C9A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="564">
   <si>
     <t>date</t>
   </si>
@@ -1706,6 +1706,12 @@
   </si>
   <si>
     <t>No. of enclaves</t>
+  </si>
+  <si>
+    <t>Word Ladder II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/word-ladder-ii/</t>
   </si>
 </sst>
 </file>
@@ -1976,7 +1982,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D281"/>
+  <dimension ref="A1:D282"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5066,6 +5072,17 @@
       </c>
       <c r="C281" s="4" t="s">
         <v>560</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A282" s="1">
+        <v>46263</v>
+      </c>
+      <c r="B282" t="s">
+        <v>562</v>
+      </c>
+      <c r="C282" s="4" t="s">
+        <v>563</v>
       </c>
     </row>
   </sheetData>
@@ -5344,8 +5361,9 @@
     <hyperlink ref="C279" r:id="rId272" xr:uid="{EE8670A5-7218-415D-ACAC-75BB144ABB37}"/>
     <hyperlink ref="C280" r:id="rId273" xr:uid="{CF717DFE-6659-495F-BFC7-5075CE2DA2EB}"/>
     <hyperlink ref="C281" r:id="rId274" xr:uid="{3AC2CD71-6543-4022-99C0-EC7F6F7C2CDE}"/>
+    <hyperlink ref="C282" r:id="rId275" xr:uid="{8F2AF890-8B0B-47DC-BDA4-868AB6C958DD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId275"/>
+  <pageSetup orientation="portrait" r:id="rId276"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem : Is Graph BiPartite
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBC68A62-C8B3-4B7C-8302-13300FA9C9A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC603795-1DD0-4442-B72D-04208CD3AAF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="566">
   <si>
     <t>date</t>
   </si>
@@ -1712,6 +1712,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/word-ladder-ii/</t>
+  </si>
+  <si>
+    <t>Bipartite Graph</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/is-graph-bipartite/</t>
   </si>
 </sst>
 </file>
@@ -1982,7 +1988,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D282"/>
+  <dimension ref="A1:D283"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5083,6 +5089,17 @@
       </c>
       <c r="C282" s="4" t="s">
         <v>563</v>
+      </c>
+    </row>
+    <row r="283" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A283" s="1">
+        <v>46267</v>
+      </c>
+      <c r="B283" t="s">
+        <v>564</v>
+      </c>
+      <c r="C283" s="4" t="s">
+        <v>565</v>
       </c>
     </row>
   </sheetData>
@@ -5362,8 +5379,9 @@
     <hyperlink ref="C280" r:id="rId273" xr:uid="{CF717DFE-6659-495F-BFC7-5075CE2DA2EB}"/>
     <hyperlink ref="C281" r:id="rId274" xr:uid="{3AC2CD71-6543-4022-99C0-EC7F6F7C2CDE}"/>
     <hyperlink ref="C282" r:id="rId275" xr:uid="{8F2AF890-8B0B-47DC-BDA4-868AB6C958DD}"/>
+    <hyperlink ref="C283" r:id="rId276" xr:uid="{5B98134F-8D7B-400B-8C85-A943D50FDD41}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId276"/>
+  <pageSetup orientation="portrait" r:id="rId277"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: find eventual safe states
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC603795-1DD0-4442-B72D-04208CD3AAF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F910FBA0-A303-44C4-8172-F51E9EDB481C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="568">
   <si>
     <t>date</t>
   </si>
@@ -1718,6 +1718,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/is-graph-bipartite/</t>
+  </si>
+  <si>
+    <t>Find Eventual Safe States</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-eventual-safe-states/</t>
   </si>
 </sst>
 </file>
@@ -1988,7 +1994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D283"/>
+  <dimension ref="A1:D284"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5100,6 +5106,17 @@
       </c>
       <c r="C283" s="4" t="s">
         <v>565</v>
+      </c>
+    </row>
+    <row r="284" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A284" s="1">
+        <v>46269</v>
+      </c>
+      <c r="B284" t="s">
+        <v>566</v>
+      </c>
+      <c r="C284" s="4" t="s">
+        <v>567</v>
       </c>
     </row>
   </sheetData>
@@ -5380,8 +5397,9 @@
     <hyperlink ref="C281" r:id="rId274" xr:uid="{3AC2CD71-6543-4022-99C0-EC7F6F7C2CDE}"/>
     <hyperlink ref="C282" r:id="rId275" xr:uid="{8F2AF890-8B0B-47DC-BDA4-868AB6C958DD}"/>
     <hyperlink ref="C283" r:id="rId276" xr:uid="{5B98134F-8D7B-400B-8C85-A943D50FDD41}"/>
+    <hyperlink ref="C284" r:id="rId277" xr:uid="{56D6B8DB-C829-42C7-B866-F6B172300E2A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId277"/>
+  <pageSetup orientation="portrait" r:id="rId278"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem : shortest path in undirected graph
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6234F94-BD2C-4A64-A6E0-E99ED360AA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B562765-E447-40BA-877B-178BB169061B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="572">
   <si>
     <t>date</t>
   </si>
@@ -1730,6 +1730,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/alien-dictionary/1</t>
+  </si>
+  <si>
+    <t>shortest path in undirected graph with unit weights from a source</t>
+  </si>
+  <si>
+    <t>https://takeuforward.org/plus/dsa/problems/shortest-path-in-undirected-graph-with-unit-weights?source=strivers-a2z-dsa-track</t>
   </si>
 </sst>
 </file>
@@ -2000,7 +2006,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D285"/>
+  <dimension ref="A1:D286"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5134,6 +5140,17 @@
       </c>
       <c r="C285" s="4" t="s">
         <v>569</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A286" s="1">
+        <v>46277</v>
+      </c>
+      <c r="B286" t="s">
+        <v>570</v>
+      </c>
+      <c r="C286" s="4" t="s">
+        <v>571</v>
       </c>
     </row>
   </sheetData>
@@ -5416,8 +5433,9 @@
     <hyperlink ref="C283" r:id="rId276" xr:uid="{5B98134F-8D7B-400B-8C85-A943D50FDD41}"/>
     <hyperlink ref="C284" r:id="rId277" xr:uid="{56D6B8DB-C829-42C7-B866-F6B172300E2A}"/>
     <hyperlink ref="C285" r:id="rId278" xr:uid="{79CA8E63-76F1-448A-9378-2093EF5ECA90}"/>
+    <hyperlink ref="C286" r:id="rId279" xr:uid="{0DF54E55-10BD-436D-A9A2-459B6EA9CA48}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId279"/>
+  <pageSetup orientation="portrait" r:id="rId280"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: shortest path in DAG
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B562765-E447-40BA-877B-178BB169061B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E890FBCE-EC20-46B8-BB43-045E8C342B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="574">
   <si>
     <t>date</t>
   </si>
@@ -1736,6 +1736,12 @@
   </si>
   <si>
     <t>https://takeuforward.org/plus/dsa/problems/shortest-path-in-undirected-graph-with-unit-weights?source=strivers-a2z-dsa-track</t>
+  </si>
+  <si>
+    <t>shortest path in DAG</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/shortest-path-in-directed-acyclic-graph/1</t>
   </si>
 </sst>
 </file>
@@ -2006,7 +2012,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D286"/>
+  <dimension ref="A1:D287"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5151,6 +5157,17 @@
       </c>
       <c r="C286" s="4" t="s">
         <v>571</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A287" s="1">
+        <v>46277</v>
+      </c>
+      <c r="B287" t="s">
+        <v>572</v>
+      </c>
+      <c r="C287" s="4" t="s">
+        <v>573</v>
       </c>
     </row>
   </sheetData>
@@ -5434,8 +5451,9 @@
     <hyperlink ref="C284" r:id="rId277" xr:uid="{56D6B8DB-C829-42C7-B866-F6B172300E2A}"/>
     <hyperlink ref="C285" r:id="rId278" xr:uid="{79CA8E63-76F1-448A-9378-2093EF5ECA90}"/>
     <hyperlink ref="C286" r:id="rId279" xr:uid="{0DF54E55-10BD-436D-A9A2-459B6EA9CA48}"/>
+    <hyperlink ref="C287" r:id="rId280" xr:uid="{BE493424-23A8-4043-BBE6-E473D0E8981F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId280"/>
+  <pageSetup orientation="portrait" r:id="rId281"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Print shortest path from src to dest in weighted undirected graph
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F95AC866-46D2-4025-B089-A1B6773E5A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58B982F0-8EF4-48B5-BE95-3610998AD418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="578">
   <si>
     <t>date</t>
   </si>
@@ -1748,6 +1748,12 @@
   </si>
   <si>
     <t>Dijkstra's Algo</t>
+  </si>
+  <si>
+    <t>Print shortest path in weighted undirected graph</t>
+  </si>
+  <si>
+    <t>https://takeuforward.org/practice/dsa/print-shortest-path-</t>
   </si>
 </sst>
 </file>
@@ -2018,7 +2024,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D288"/>
+  <dimension ref="A1:D289"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5185,6 +5191,17 @@
       </c>
       <c r="C288" s="4" t="s">
         <v>574</v>
+      </c>
+    </row>
+    <row r="289" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A289" s="1">
+        <v>46288</v>
+      </c>
+      <c r="B289" t="s">
+        <v>576</v>
+      </c>
+      <c r="C289" s="4" t="s">
+        <v>577</v>
       </c>
     </row>
   </sheetData>
@@ -5470,8 +5487,9 @@
     <hyperlink ref="C286" r:id="rId279" xr:uid="{0DF54E55-10BD-436D-A9A2-459B6EA9CA48}"/>
     <hyperlink ref="C287" r:id="rId280" xr:uid="{BE493424-23A8-4043-BBE6-E473D0E8981F}"/>
     <hyperlink ref="C288" r:id="rId281" xr:uid="{EF481D6B-C283-4D84-BCB3-1C5A82FC4092}"/>
+    <hyperlink ref="C289" r:id="rId282" xr:uid="{B851F673-F9A0-4E3B-8BDD-670563A935F5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId282"/>
+  <pageSetup orientation="portrait" r:id="rId283"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Shortes path in binary maze and codevita problem
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58B982F0-8EF4-48B5-BE95-3610998AD418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B0BF4B-8D4D-4AF6-833A-3789EA50106F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="580">
   <si>
     <t>date</t>
   </si>
@@ -1754,6 +1754,12 @@
   </si>
   <si>
     <t>https://takeuforward.org/practice/dsa/print-shortest-path-</t>
+  </si>
+  <si>
+    <t>Shortest Path in binary maze</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/shortest-path-in-a-binary-maze-1655453161/1</t>
   </si>
 </sst>
 </file>
@@ -2024,7 +2030,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D289"/>
+  <dimension ref="A1:D290"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5202,6 +5208,17 @@
       </c>
       <c r="C289" s="4" t="s">
         <v>577</v>
+      </c>
+    </row>
+    <row r="290" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A290" s="1">
+        <v>46289</v>
+      </c>
+      <c r="B290" t="s">
+        <v>578</v>
+      </c>
+      <c r="C290" s="4" t="s">
+        <v>579</v>
       </c>
     </row>
   </sheetData>
@@ -5488,8 +5505,9 @@
     <hyperlink ref="C287" r:id="rId280" xr:uid="{BE493424-23A8-4043-BBE6-E473D0E8981F}"/>
     <hyperlink ref="C288" r:id="rId281" xr:uid="{EF481D6B-C283-4D84-BCB3-1C5A82FC4092}"/>
     <hyperlink ref="C289" r:id="rId282" xr:uid="{B851F673-F9A0-4E3B-8BDD-670563A935F5}"/>
+    <hyperlink ref="C290" r:id="rId283" xr:uid="{8975C409-FB81-4588-8765-D282BDDE9C60}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId283"/>
+  <pageSetup orientation="portrait" r:id="rId284"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: Path with minimum effort
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B0BF4B-8D4D-4AF6-833A-3789EA50106F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4FCF56D-15E8-48A1-AEFF-D88A70F5A1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="582">
   <si>
     <t>date</t>
   </si>
@@ -1760,6 +1760,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/shortest-path-in-a-binary-maze-1655453161/1</t>
+  </si>
+  <si>
+    <t>path with min. effort</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/path-with-minimum-effort/</t>
   </si>
 </sst>
 </file>
@@ -2030,7 +2036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D290"/>
+  <dimension ref="A1:D291"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5219,6 +5225,17 @@
       </c>
       <c r="C290" s="4" t="s">
         <v>579</v>
+      </c>
+    </row>
+    <row r="291" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A291" s="1">
+        <v>46291</v>
+      </c>
+      <c r="B291" t="s">
+        <v>580</v>
+      </c>
+      <c r="C291" s="4" t="s">
+        <v>581</v>
       </c>
     </row>
   </sheetData>
@@ -5506,8 +5523,9 @@
     <hyperlink ref="C288" r:id="rId281" xr:uid="{EF481D6B-C283-4D84-BCB3-1C5A82FC4092}"/>
     <hyperlink ref="C289" r:id="rId282" xr:uid="{B851F673-F9A0-4E3B-8BDD-670563A935F5}"/>
     <hyperlink ref="C290" r:id="rId283" xr:uid="{8975C409-FB81-4588-8765-D282BDDE9C60}"/>
+    <hyperlink ref="C291" r:id="rId284" xr:uid="{EF8A9816-EDB7-418B-BFEC-733EB49E7D71}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId284"/>
+  <pageSetup orientation="portrait" r:id="rId285"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem : cheapest flights within k steps
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4FCF56D-15E8-48A1-AEFF-D88A70F5A1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33BCA1D8-7E20-4A18-8F03-0C8380033AD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="582">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="584">
   <si>
     <t>date</t>
   </si>
@@ -1766,6 +1766,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/path-with-minimum-effort/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/cheapest-flights-within-k-stops/</t>
+  </si>
+  <si>
+    <t>cheapest flights with k stops</t>
   </si>
 </sst>
 </file>
@@ -2036,7 +2042,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D291"/>
+  <dimension ref="A1:D292"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5236,6 +5242,17 @@
       </c>
       <c r="C291" s="4" t="s">
         <v>581</v>
+      </c>
+    </row>
+    <row r="292" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A292" s="1">
+        <v>46294</v>
+      </c>
+      <c r="B292" t="s">
+        <v>583</v>
+      </c>
+      <c r="C292" s="4" t="s">
+        <v>582</v>
       </c>
     </row>
   </sheetData>
@@ -5524,8 +5541,9 @@
     <hyperlink ref="C289" r:id="rId282" xr:uid="{B851F673-F9A0-4E3B-8BDD-670563A935F5}"/>
     <hyperlink ref="C290" r:id="rId283" xr:uid="{8975C409-FB81-4588-8765-D282BDDE9C60}"/>
     <hyperlink ref="C291" r:id="rId284" xr:uid="{EF8A9816-EDB7-418B-BFEC-733EB49E7D71}"/>
+    <hyperlink ref="C292" r:id="rId285" xr:uid="{69B62C10-D6AD-407A-8069-D30E71EBC5B5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId285"/>
+  <pageSetup orientation="portrait" r:id="rId286"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: min. multiplications to reach end
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33BCA1D8-7E20-4A18-8F03-0C8380033AD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7FA7535-1CC2-4BCA-B56E-9A816DAEEBAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="586">
   <si>
     <t>date</t>
   </si>
@@ -1772,6 +1772,12 @@
   </si>
   <si>
     <t>cheapest flights with k stops</t>
+  </si>
+  <si>
+    <t>min. multiplications to reach end</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/minimum-multiplications-to-reach-end/1</t>
   </si>
 </sst>
 </file>
@@ -2042,7 +2048,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D292"/>
+  <dimension ref="A1:D293"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5253,6 +5259,17 @@
       </c>
       <c r="C292" s="4" t="s">
         <v>582</v>
+      </c>
+    </row>
+    <row r="293" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A293" s="1">
+        <v>46295</v>
+      </c>
+      <c r="B293" t="s">
+        <v>584</v>
+      </c>
+      <c r="C293" s="4" t="s">
+        <v>585</v>
       </c>
     </row>
   </sheetData>
@@ -5542,8 +5559,9 @@
     <hyperlink ref="C290" r:id="rId283" xr:uid="{8975C409-FB81-4588-8765-D282BDDE9C60}"/>
     <hyperlink ref="C291" r:id="rId284" xr:uid="{EF8A9816-EDB7-418B-BFEC-733EB49E7D71}"/>
     <hyperlink ref="C292" r:id="rId285" xr:uid="{69B62C10-D6AD-407A-8069-D30E71EBC5B5}"/>
+    <hyperlink ref="C293" r:id="rId286" xr:uid="{F9AAF73A-EAA5-4A21-9101-9E392060C64F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId286"/>
+  <pageSetup orientation="portrait" r:id="rId287"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: no. of ways to arrive at destination
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7FA7535-1CC2-4BCA-B56E-9A816DAEEBAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B418A72-9EB6-4B36-8DE6-D8590BE2F91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="586">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="588">
   <si>
     <t>date</t>
   </si>
@@ -1778,6 +1778,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/minimum-multiplications-to-reach-end/1</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/number-of-ways-to-arrive-at-destination/</t>
+  </si>
+  <si>
+    <t>No. of ways to arrive at destination</t>
   </si>
 </sst>
 </file>
@@ -2048,7 +2054,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D293"/>
+  <dimension ref="A1:D294"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5270,6 +5276,17 @@
       </c>
       <c r="C293" s="4" t="s">
         <v>585</v>
+      </c>
+    </row>
+    <row r="294" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A294" s="1">
+        <v>46296</v>
+      </c>
+      <c r="B294" t="s">
+        <v>587</v>
+      </c>
+      <c r="C294" s="4" t="s">
+        <v>586</v>
       </c>
     </row>
   </sheetData>
@@ -5560,8 +5577,9 @@
     <hyperlink ref="C291" r:id="rId284" xr:uid="{EF8A9816-EDB7-418B-BFEC-733EB49E7D71}"/>
     <hyperlink ref="C292" r:id="rId285" xr:uid="{69B62C10-D6AD-407A-8069-D30E71EBC5B5}"/>
     <hyperlink ref="C293" r:id="rId286" xr:uid="{F9AAF73A-EAA5-4A21-9101-9E392060C64F}"/>
+    <hyperlink ref="C294" r:id="rId287" xr:uid="{9FED40AF-456F-4709-AF2C-20670678F914}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId287"/>
+  <pageSetup orientation="portrait" r:id="rId288"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: Bellman Ford Algo
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B418A72-9EB6-4B36-8DE6-D8590BE2F91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD82568F-9101-434D-9D8A-37F6AC148D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="590">
   <si>
     <t>date</t>
   </si>
@@ -1784,6 +1784,12 @@
   </si>
   <si>
     <t>No. of ways to arrive at destination</t>
+  </si>
+  <si>
+    <t>Bellman-Ford Algo</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/distance-from-the-source-bellman-ford-algorithm/1</t>
   </si>
 </sst>
 </file>
@@ -2054,7 +2060,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D294"/>
+  <dimension ref="A1:D295"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5287,6 +5293,17 @@
       </c>
       <c r="C294" s="4" t="s">
         <v>586</v>
+      </c>
+    </row>
+    <row r="295" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A295" s="1">
+        <v>46297</v>
+      </c>
+      <c r="B295" t="s">
+        <v>588</v>
+      </c>
+      <c r="C295" s="4" t="s">
+        <v>589</v>
       </c>
     </row>
   </sheetData>
@@ -5578,8 +5595,9 @@
     <hyperlink ref="C292" r:id="rId285" xr:uid="{69B62C10-D6AD-407A-8069-D30E71EBC5B5}"/>
     <hyperlink ref="C293" r:id="rId286" xr:uid="{F9AAF73A-EAA5-4A21-9101-9E392060C64F}"/>
     <hyperlink ref="C294" r:id="rId287" xr:uid="{9FED40AF-456F-4709-AF2C-20670678F914}"/>
+    <hyperlink ref="C295" r:id="rId288" xr:uid="{B80A9E9F-6E46-4C60-A84F-BFBF9AB8CA01}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId288"/>
+  <pageSetup orientation="portrait" r:id="rId289"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: no. of cities with smallest no. of neighbours within threshold dist.
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD82568F-9101-434D-9D8A-37F6AC148D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AB1A2F6-7CE7-4C9C-8405-BDDF9071D3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="592">
   <si>
     <t>date</t>
   </si>
@@ -1790,6 +1790,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/distance-from-the-source-bellman-ford-algorithm/1</t>
+  </si>
+  <si>
+    <t>Find the city with smallest no. of nodes within threshold distance</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-the-city-with-the-smallest-number-of-neighbors-at-a-threshold-distance/</t>
   </si>
 </sst>
 </file>
@@ -2060,7 +2066,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D295"/>
+  <dimension ref="A1:D296"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5304,6 +5310,17 @@
       </c>
       <c r="C295" s="4" t="s">
         <v>589</v>
+      </c>
+    </row>
+    <row r="296" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A296" s="1">
+        <v>46303</v>
+      </c>
+      <c r="B296" t="s">
+        <v>590</v>
+      </c>
+      <c r="C296" s="4" t="s">
+        <v>591</v>
       </c>
     </row>
   </sheetData>
@@ -5596,8 +5613,9 @@
     <hyperlink ref="C293" r:id="rId286" xr:uid="{F9AAF73A-EAA5-4A21-9101-9E392060C64F}"/>
     <hyperlink ref="C294" r:id="rId287" xr:uid="{9FED40AF-456F-4709-AF2C-20670678F914}"/>
     <hyperlink ref="C295" r:id="rId288" xr:uid="{B80A9E9F-6E46-4C60-A84F-BFBF9AB8CA01}"/>
+    <hyperlink ref="C296" r:id="rId289" xr:uid="{A8EFDD05-7A08-43EE-A279-70A8A0765E53}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId289"/>
+  <pageSetup orientation="portrait" r:id="rId290"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: network delay time
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AB1A2F6-7CE7-4C9C-8405-BDDF9071D3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481A63BE-2308-485F-A146-FA5E84A37424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="594">
   <si>
     <t>date</t>
   </si>
@@ -1796,6 +1796,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/find-the-city-with-the-smallest-number-of-neighbors-at-a-threshold-distance/</t>
+  </si>
+  <si>
+    <t>Network Delay Time</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/network-delay-time/</t>
   </si>
 </sst>
 </file>
@@ -2066,7 +2072,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D296"/>
+  <dimension ref="A1:D297"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5321,6 +5327,17 @@
       </c>
       <c r="C296" s="4" t="s">
         <v>591</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A297" s="1">
+        <v>46304</v>
+      </c>
+      <c r="B297" t="s">
+        <v>592</v>
+      </c>
+      <c r="C297" s="4" t="s">
+        <v>593</v>
       </c>
     </row>
   </sheetData>
@@ -5614,8 +5631,9 @@
     <hyperlink ref="C294" r:id="rId287" xr:uid="{9FED40AF-456F-4709-AF2C-20670678F914}"/>
     <hyperlink ref="C295" r:id="rId288" xr:uid="{B80A9E9F-6E46-4C60-A84F-BFBF9AB8CA01}"/>
     <hyperlink ref="C296" r:id="rId289" xr:uid="{A8EFDD05-7A08-43EE-A279-70A8A0765E53}"/>
+    <hyperlink ref="C297" r:id="rId290" xr:uid="{BDAB10DE-99E5-48B3-BDA3-E2C3F12DB597}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId290"/>
+  <pageSetup orientation="portrait" r:id="rId291"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: swim in rising water
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481A63BE-2308-485F-A146-FA5E84A37424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9C9F20D-A7ED-422A-9BF6-F10173775E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="594">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="596">
   <si>
     <t>date</t>
   </si>
@@ -1802,6 +1802,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/network-delay-time/</t>
+  </si>
+  <si>
+    <t>Swim in rising water</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/swim-in-rising-water/</t>
   </si>
 </sst>
 </file>
@@ -2072,7 +2078,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D297"/>
+  <dimension ref="A1:D298"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5338,6 +5344,17 @@
       </c>
       <c r="C297" s="4" t="s">
         <v>593</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A298" s="1">
+        <v>46305</v>
+      </c>
+      <c r="B298" t="s">
+        <v>594</v>
+      </c>
+      <c r="C298" s="4" t="s">
+        <v>595</v>
       </c>
     </row>
   </sheetData>
@@ -5632,8 +5649,9 @@
     <hyperlink ref="C295" r:id="rId288" xr:uid="{B80A9E9F-6E46-4C60-A84F-BFBF9AB8CA01}"/>
     <hyperlink ref="C296" r:id="rId289" xr:uid="{A8EFDD05-7A08-43EE-A279-70A8A0765E53}"/>
     <hyperlink ref="C297" r:id="rId290" xr:uid="{BDAB10DE-99E5-48B3-BDA3-E2C3F12DB597}"/>
+    <hyperlink ref="C298" r:id="rId291" xr:uid="{AACDA2B1-D222-4119-8510-76C57919578E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId291"/>
+  <pageSetup orientation="portrait" r:id="rId292"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Many POTD are solved
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9C9F20D-A7ED-422A-9BF6-F10173775E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5621BB1-5EBF-4E9F-AE1E-4EC45BC4F3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="604">
   <si>
     <t>date</t>
   </si>
@@ -1808,6 +1808,30 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/swim-in-rising-water/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximum-alternating-sum-of-squares/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximize-sum-of-squares-of-digits</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/subarrays-distinct-element-sum-of-squares-i/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-swaps-to-sort-by-digit-sum/</t>
+  </si>
+  <si>
+    <t>Max. alternating sum of squares</t>
+  </si>
+  <si>
+    <t>maximize sum of square of digits</t>
+  </si>
+  <si>
+    <t>subarrays distinct element sum of squares I</t>
+  </si>
+  <si>
+    <t>min. swaps to sort by digit sum</t>
   </si>
 </sst>
 </file>
@@ -2078,7 +2102,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D298"/>
+  <dimension ref="A1:D302"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5355,6 +5379,50 @@
       </c>
       <c r="C298" s="4" t="s">
         <v>595</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A299" s="1">
+        <v>46308</v>
+      </c>
+      <c r="B299" t="s">
+        <v>600</v>
+      </c>
+      <c r="C299" s="4" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A300" s="1">
+        <v>46309</v>
+      </c>
+      <c r="B300" t="s">
+        <v>601</v>
+      </c>
+      <c r="C300" s="4" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A301" s="1">
+        <v>46310</v>
+      </c>
+      <c r="B301" t="s">
+        <v>602</v>
+      </c>
+      <c r="C301" s="4" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A302" s="1">
+        <v>46312</v>
+      </c>
+      <c r="B302" t="s">
+        <v>603</v>
+      </c>
+      <c r="C302" s="4" t="s">
+        <v>599</v>
       </c>
     </row>
   </sheetData>
@@ -5650,8 +5718,12 @@
     <hyperlink ref="C296" r:id="rId289" xr:uid="{A8EFDD05-7A08-43EE-A279-70A8A0765E53}"/>
     <hyperlink ref="C297" r:id="rId290" xr:uid="{BDAB10DE-99E5-48B3-BDA3-E2C3F12DB597}"/>
     <hyperlink ref="C298" r:id="rId291" xr:uid="{AACDA2B1-D222-4119-8510-76C57919578E}"/>
+    <hyperlink ref="C299" r:id="rId292" xr:uid="{32DEFC19-293E-4182-B58F-085C76323A63}"/>
+    <hyperlink ref="C300" r:id="rId293" xr:uid="{BE3937EA-3F02-4F46-834F-27F8EA1BB5C1}"/>
+    <hyperlink ref="C301" r:id="rId294" xr:uid="{DE7AD2E7-C605-4CF1-A3D3-93197A821E13}"/>
+    <hyperlink ref="C302" r:id="rId295" xr:uid="{BC230DCC-643F-4D44-8514-14FF78590274}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId292"/>
+  <pageSetup orientation="portrait" r:id="rId296"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
no. of operations to make network connected
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5621BB1-5EBF-4E9F-AE1E-4EC45BC4F3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449F15DF-DFF6-48B9-BA68-1B6C08A04778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="604">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="606">
   <si>
     <t>date</t>
   </si>
@@ -1832,6 +1832,12 @@
   </si>
   <si>
     <t>min. swaps to sort by digit sum</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/number-of-operations-to-make-network-connected/</t>
+  </si>
+  <si>
+    <t>no. of operations to make network connected</t>
   </si>
 </sst>
 </file>
@@ -2102,7 +2108,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D302"/>
+  <dimension ref="A1:D303"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5423,6 +5429,17 @@
       </c>
       <c r="C302" s="4" t="s">
         <v>599</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A303" s="1">
+        <v>46312</v>
+      </c>
+      <c r="B303" t="s">
+        <v>605</v>
+      </c>
+      <c r="C303" s="4" t="s">
+        <v>604</v>
       </c>
     </row>
   </sheetData>
@@ -5722,8 +5739,9 @@
     <hyperlink ref="C300" r:id="rId293" xr:uid="{BE3937EA-3F02-4F46-834F-27F8EA1BB5C1}"/>
     <hyperlink ref="C301" r:id="rId294" xr:uid="{DE7AD2E7-C605-4CF1-A3D3-93197A821E13}"/>
     <hyperlink ref="C302" r:id="rId295" xr:uid="{BC230DCC-643F-4D44-8514-14FF78590274}"/>
+    <hyperlink ref="C303" r:id="rId296" xr:uid="{737043F5-19A9-433C-8827-EE0547800701}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId296"/>
+  <pageSetup orientation="portrait" r:id="rId297"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: range sum query
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449F15DF-DFF6-48B9-BA68-1B6C08A04778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEBC8B81-09AD-4645-A2C4-743B32A66F7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="606">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="610">
   <si>
     <t>date</t>
   </si>
@@ -1838,6 +1838,18 @@
   </si>
   <si>
     <t>no. of operations to make network connected</t>
+  </si>
+  <si>
+    <t>range sum query immutable</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/range-sum-query-immutable/</t>
+  </si>
+  <si>
+    <t>range sum query mutable</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/range-sum-query-mutable/</t>
   </si>
 </sst>
 </file>
@@ -2108,7 +2120,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D303"/>
+  <dimension ref="A1:D305"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5440,6 +5452,28 @@
       </c>
       <c r="C303" s="4" t="s">
         <v>604</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A304" s="1">
+        <v>46312</v>
+      </c>
+      <c r="B304" t="s">
+        <v>606</v>
+      </c>
+      <c r="C304" s="4" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A305" s="1">
+        <v>46312</v>
+      </c>
+      <c r="B305" t="s">
+        <v>608</v>
+      </c>
+      <c r="C305" s="4" t="s">
+        <v>609</v>
       </c>
     </row>
   </sheetData>
@@ -5740,8 +5774,10 @@
     <hyperlink ref="C301" r:id="rId294" xr:uid="{DE7AD2E7-C605-4CF1-A3D3-93197A821E13}"/>
     <hyperlink ref="C302" r:id="rId295" xr:uid="{BC230DCC-643F-4D44-8514-14FF78590274}"/>
     <hyperlink ref="C303" r:id="rId296" xr:uid="{737043F5-19A9-433C-8827-EE0547800701}"/>
+    <hyperlink ref="C304" r:id="rId297" xr:uid="{4543DD75-2A6B-46F6-AA4B-04B95C75062E}"/>
+    <hyperlink ref="C305" r:id="rId298" xr:uid="{05A8CDB8-DDB2-4089-9A70-11DCDED824F1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId297"/>
+  <pageSetup orientation="portrait" r:id="rId299"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: min. opns to sort a permutation
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEBC8B81-09AD-4645-A2C4-743B32A66F7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{028CB4EA-2035-40D1-AB71-0FC9062501DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="610">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="612">
   <si>
     <t>date</t>
   </si>
@@ -1850,6 +1850,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/range-sum-query-mutable/</t>
+  </si>
+  <si>
+    <t>min. operations to sort a permutation</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-operations-to-sort-a-permutation/</t>
   </si>
 </sst>
 </file>
@@ -2120,7 +2126,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D305"/>
+  <dimension ref="A1:D306"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5474,6 +5480,17 @@
       </c>
       <c r="C305" s="4" t="s">
         <v>609</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A306" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B306" t="s">
+        <v>610</v>
+      </c>
+      <c r="C306" s="4" t="s">
+        <v>611</v>
       </c>
     </row>
   </sheetData>
@@ -5776,8 +5793,9 @@
     <hyperlink ref="C303" r:id="rId296" xr:uid="{737043F5-19A9-433C-8827-EE0547800701}"/>
     <hyperlink ref="C304" r:id="rId297" xr:uid="{4543DD75-2A6B-46F6-AA4B-04B95C75062E}"/>
     <hyperlink ref="C305" r:id="rId298" xr:uid="{05A8CDB8-DDB2-4089-9A70-11DCDED824F1}"/>
+    <hyperlink ref="C306" r:id="rId299" xr:uid="{60EDDC09-8C66-490D-A7C2-7ECD02B7C88A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId299"/>
+  <pageSetup orientation="portrait" r:id="rId300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: range min. query
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5FB6E7C-45B3-4E4C-BEEA-1A7E90424079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511DC6C6-1EAD-4AA2-88E7-B807409E3ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="616">
   <si>
     <t>date</t>
   </si>
@@ -1862,6 +1862,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/accounts-merge/</t>
+  </si>
+  <si>
+    <t>range min. query</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/range-minimum-query/1</t>
   </si>
 </sst>
 </file>
@@ -2132,7 +2138,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D307"/>
+  <dimension ref="A1:D308"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5508,6 +5514,17 @@
       </c>
       <c r="C307" s="4" t="s">
         <v>613</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A308" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B308" t="s">
+        <v>614</v>
+      </c>
+      <c r="C308" s="4" t="s">
+        <v>615</v>
       </c>
     </row>
   </sheetData>
@@ -5812,8 +5829,9 @@
     <hyperlink ref="C305" r:id="rId298" xr:uid="{05A8CDB8-DDB2-4089-9A70-11DCDED824F1}"/>
     <hyperlink ref="C306" r:id="rId299" xr:uid="{60EDDC09-8C66-490D-A7C2-7ECD02B7C88A}"/>
     <hyperlink ref="C307" r:id="rId300" xr:uid="{BF2CD767-F74C-42C1-9CCE-E764DD0EDFB5}"/>
+    <hyperlink ref="C308" r:id="rId301" xr:uid="{B203D168-AE68-4649-A053-C669B29F8E8C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId301"/>
+  <pageSetup orientation="portrait" r:id="rId302"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: count no of days together
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511DC6C6-1EAD-4AA2-88E7-B807409E3ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4082C259-F18A-4A73-8D57-E48EE6E1933B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="618">
   <si>
     <t>date</t>
   </si>
@@ -1868,6 +1868,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/range-minimum-query/1</t>
+  </si>
+  <si>
+    <t>count days spent together</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/count-days-spent-together/</t>
   </si>
 </sst>
 </file>
@@ -2138,7 +2144,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D308"/>
+  <dimension ref="A1:D309"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5525,6 +5531,17 @@
       </c>
       <c r="C308" s="4" t="s">
         <v>615</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A309" s="1">
+        <v>46319</v>
+      </c>
+      <c r="B309" t="s">
+        <v>616</v>
+      </c>
+      <c r="C309" s="4" t="s">
+        <v>617</v>
       </c>
     </row>
   </sheetData>
@@ -5830,8 +5847,9 @@
     <hyperlink ref="C306" r:id="rId299" xr:uid="{60EDDC09-8C66-490D-A7C2-7ECD02B7C88A}"/>
     <hyperlink ref="C307" r:id="rId300" xr:uid="{BF2CD767-F74C-42C1-9CCE-E764DD0EDFB5}"/>
     <hyperlink ref="C308" r:id="rId301" xr:uid="{B203D168-AE68-4649-A053-C669B29F8E8C}"/>
+    <hyperlink ref="C309" r:id="rId302" xr:uid="{63D7FF21-E247-4E90-9578-FD056EEDC88C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId302"/>
+  <pageSetup orientation="portrait" r:id="rId303"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
problem: no. of islands II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4082C259-F18A-4A73-8D57-E48EE6E1933B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{456FCFAD-E4CB-4D9C-84C8-3B6140742D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="620">
   <si>
     <t>date</t>
   </si>
@@ -1874,6 +1874,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/count-days-spent-together/</t>
+  </si>
+  <si>
+    <t>number of islands II</t>
+  </si>
+  <si>
+    <t>https://www.naukri.com/code360/problems/number-of-islands-ii_1266048?leftPanelTabValue=PROBLEM</t>
   </si>
 </sst>
 </file>
@@ -2144,7 +2150,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D309"/>
+  <dimension ref="A1:D310"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5542,6 +5548,17 @@
       </c>
       <c r="C309" s="4" t="s">
         <v>617</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A310" s="1">
+        <v>46320</v>
+      </c>
+      <c r="B310" t="s">
+        <v>618</v>
+      </c>
+      <c r="C310" s="4" t="s">
+        <v>619</v>
       </c>
     </row>
   </sheetData>
@@ -5848,8 +5865,9 @@
     <hyperlink ref="C307" r:id="rId300" xr:uid="{BF2CD767-F74C-42C1-9CCE-E764DD0EDFB5}"/>
     <hyperlink ref="C308" r:id="rId301" xr:uid="{B203D168-AE68-4649-A053-C669B29F8E8C}"/>
     <hyperlink ref="C309" r:id="rId302" xr:uid="{63D7FF21-E247-4E90-9578-FD056EEDC88C}"/>
+    <hyperlink ref="C310" r:id="rId303" xr:uid="{5B221B5E-45E0-4760-B49A-9422FF316119}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId303"/>
+  <pageSetup orientation="portrait" r:id="rId304"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
making a large island and no. of closed islands
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{456FCFAD-E4CB-4D9C-84C8-3B6140742D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{438C89B8-8686-490D-9BA1-47264F266DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="624">
   <si>
     <t>date</t>
   </si>
@@ -1880,6 +1880,18 @@
   </si>
   <si>
     <t>https://www.naukri.com/code360/problems/number-of-islands-ii_1266048?leftPanelTabValue=PROBLEM</t>
+  </si>
+  <si>
+    <t>number of closed islands</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/number-of-closed-islands/</t>
+  </si>
+  <si>
+    <t>making a large island</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/making-a-large-island/</t>
   </si>
 </sst>
 </file>
@@ -2150,7 +2162,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D310"/>
+  <dimension ref="A1:D312"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5559,6 +5571,28 @@
       </c>
       <c r="C310" s="4" t="s">
         <v>619</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A311" s="1">
+        <v>46320</v>
+      </c>
+      <c r="B311" t="s">
+        <v>620</v>
+      </c>
+      <c r="C311" s="4" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A312" s="1">
+        <v>46320</v>
+      </c>
+      <c r="B312" t="s">
+        <v>622</v>
+      </c>
+      <c r="C312" s="4" t="s">
+        <v>623</v>
       </c>
     </row>
   </sheetData>
@@ -5866,8 +5900,10 @@
     <hyperlink ref="C308" r:id="rId301" xr:uid="{B203D168-AE68-4649-A053-C669B29F8E8C}"/>
     <hyperlink ref="C309" r:id="rId302" xr:uid="{63D7FF21-E247-4E90-9578-FD056EEDC88C}"/>
     <hyperlink ref="C310" r:id="rId303" xr:uid="{5B221B5E-45E0-4760-B49A-9422FF316119}"/>
+    <hyperlink ref="C311" r:id="rId304" xr:uid="{2D94045C-2F84-4B60-990A-DF65C1B05B87}"/>
+    <hyperlink ref="C312" r:id="rId305" xr:uid="{30D414F1-AB03-49CF-864B-C3E0D887C46A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId304"/>
+  <pageSetup orientation="portrait" r:id="rId306"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: count islands with total value divisible by k
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{438C89B8-8686-490D-9BA1-47264F266DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D3D3B80-38D1-4D9C-B77F-D34F78579E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="626">
   <si>
     <t>date</t>
   </si>
@@ -1892,6 +1892,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/making-a-large-island/</t>
+  </si>
+  <si>
+    <t>count islands with total value divisible by k</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/count-islands-with-total-value-divisible-by-k/</t>
   </si>
 </sst>
 </file>
@@ -2162,7 +2168,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D312"/>
+  <dimension ref="A1:D313"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5593,6 +5599,17 @@
       </c>
       <c r="C312" s="4" t="s">
         <v>623</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A313" s="1">
+        <v>46321</v>
+      </c>
+      <c r="B313" t="s">
+        <v>624</v>
+      </c>
+      <c r="C313" s="4" t="s">
+        <v>625</v>
       </c>
     </row>
   </sheetData>
@@ -5902,8 +5919,9 @@
     <hyperlink ref="C310" r:id="rId303" xr:uid="{5B221B5E-45E0-4760-B49A-9422FF316119}"/>
     <hyperlink ref="C311" r:id="rId304" xr:uid="{2D94045C-2F84-4B60-990A-DF65C1B05B87}"/>
     <hyperlink ref="C312" r:id="rId305" xr:uid="{30D414F1-AB03-49CF-864B-C3E0D887C46A}"/>
+    <hyperlink ref="C313" r:id="rId306" xr:uid="{9D51E31B-9F33-4614-B047-4FA8E61E9A74}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId306"/>
+  <pageSetup orientation="portrait" r:id="rId307"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: most stones removed from same row or column
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D3D3B80-38D1-4D9C-B77F-D34F78579E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6340E1B6-CCFA-4504-ABBE-04395DB0E4A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="626">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="628">
   <si>
     <t>date</t>
   </si>
@@ -1898,6 +1898,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/count-islands-with-total-value-divisible-by-k/</t>
+  </si>
+  <si>
+    <t>most stones removed with same row or column</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/most-stones-removed-with-same-row-or-column/</t>
   </si>
 </sst>
 </file>
@@ -2168,7 +2174,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D313"/>
+  <dimension ref="A1:D314"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5610,6 +5616,17 @@
       </c>
       <c r="C313" s="4" t="s">
         <v>625</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A314" s="1">
+        <v>46321</v>
+      </c>
+      <c r="B314" t="s">
+        <v>626</v>
+      </c>
+      <c r="C314" s="4" t="s">
+        <v>627</v>
       </c>
     </row>
   </sheetData>
@@ -5920,8 +5937,9 @@
     <hyperlink ref="C311" r:id="rId304" xr:uid="{2D94045C-2F84-4B60-990A-DF65C1B05B87}"/>
     <hyperlink ref="C312" r:id="rId305" xr:uid="{30D414F1-AB03-49CF-864B-C3E0D887C46A}"/>
     <hyperlink ref="C313" r:id="rId306" xr:uid="{9D51E31B-9F33-4614-B047-4FA8E61E9A74}"/>
+    <hyperlink ref="C314" r:id="rId307" xr:uid="{B3935C31-E87D-44D7-AFAB-FACA45F44114}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId307"/>
+  <pageSetup orientation="portrait" r:id="rId308"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: subArrays distinct element sum of squares II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6340E1B6-CCFA-4504-ABBE-04395DB0E4A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADBB72B-51C2-4842-BC86-7AF7D58361CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="628">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="630">
   <si>
     <t>date</t>
   </si>
@@ -1904,6 +1904,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/most-stones-removed-with-same-row-or-column/</t>
+  </si>
+  <si>
+    <t>subarrays distinct element sum of squares II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/subarrays-distinct-element-sum-of-squares-ii/</t>
   </si>
 </sst>
 </file>
@@ -2174,7 +2180,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D314"/>
+  <dimension ref="A1:D315"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5627,6 +5633,17 @@
       </c>
       <c r="C314" s="4" t="s">
         <v>627</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A315" s="1">
+        <v>46321</v>
+      </c>
+      <c r="B315" t="s">
+        <v>628</v>
+      </c>
+      <c r="C315" s="4" t="s">
+        <v>629</v>
       </c>
     </row>
   </sheetData>
@@ -5938,8 +5955,9 @@
     <hyperlink ref="C312" r:id="rId305" xr:uid="{30D414F1-AB03-49CF-864B-C3E0D887C46A}"/>
     <hyperlink ref="C313" r:id="rId306" xr:uid="{9D51E31B-9F33-4614-B047-4FA8E61E9A74}"/>
     <hyperlink ref="C314" r:id="rId307" xr:uid="{B3935C31-E87D-44D7-AFAB-FACA45F44114}"/>
+    <hyperlink ref="C315" r:id="rId308" xr:uid="{F0BA794F-8B1E-4F8D-BC01-FF39F7A2861F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId308"/>
+  <pageSetup orientation="portrait" r:id="rId309"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: create grid with exactly one path
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADBB72B-51C2-4842-BC86-7AF7D58361CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F67E8256-884E-4E28-9D7E-F5D21219C3C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="632">
   <si>
     <t>date</t>
   </si>
@@ -1910,6 +1910,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/subarrays-distinct-element-sum-of-squares-ii/</t>
+  </si>
+  <si>
+    <t>create grid with exactly one path</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/create-grid-with-exactly-one-path/</t>
   </si>
 </sst>
 </file>
@@ -2180,7 +2186,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D315"/>
+  <dimension ref="A1:D316"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5644,6 +5650,17 @@
       </c>
       <c r="C315" s="4" t="s">
         <v>629</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A316" s="1">
+        <v>46322</v>
+      </c>
+      <c r="B316" t="s">
+        <v>630</v>
+      </c>
+      <c r="C316" s="4" t="s">
+        <v>631</v>
       </c>
     </row>
   </sheetData>
@@ -5956,8 +5973,9 @@
     <hyperlink ref="C313" r:id="rId306" xr:uid="{9D51E31B-9F33-4614-B047-4FA8E61E9A74}"/>
     <hyperlink ref="C314" r:id="rId307" xr:uid="{B3935C31-E87D-44D7-AFAB-FACA45F44114}"/>
     <hyperlink ref="C315" r:id="rId308" xr:uid="{F0BA794F-8B1E-4F8D-BC01-FF39F7A2861F}"/>
+    <hyperlink ref="C316" r:id="rId309" xr:uid="{408E3341-8CF0-4E72-B1CF-BE0BC4E6103E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId309"/>
+  <pageSetup orientation="portrait" r:id="rId310"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: min. XOR path in a grid(DP)
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BBD49D7-D3EC-437C-8EA0-5277AB813A9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{581D649E-C25D-4EAB-9BF6-EBFFB3D0C971}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="634">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="636">
   <si>
     <t>date</t>
   </si>
@@ -1922,6 +1922,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/strongly-connected-components-kosarajus-algo/1</t>
+  </si>
+  <si>
+    <t>min. xor path in a grid</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-xor-path-in-a-grid/</t>
   </si>
 </sst>
 </file>
@@ -2192,7 +2198,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D317"/>
+  <dimension ref="A1:D318"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5678,6 +5684,17 @@
       </c>
       <c r="C317" s="4" t="s">
         <v>633</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A318" s="1">
+        <v>46323</v>
+      </c>
+      <c r="B318" t="s">
+        <v>634</v>
+      </c>
+      <c r="C318" s="4" t="s">
+        <v>635</v>
       </c>
     </row>
   </sheetData>
@@ -5992,8 +6009,9 @@
     <hyperlink ref="C315" r:id="rId308" xr:uid="{F0BA794F-8B1E-4F8D-BC01-FF39F7A2861F}"/>
     <hyperlink ref="C316" r:id="rId309" xr:uid="{408E3341-8CF0-4E72-B1CF-BE0BC4E6103E}"/>
     <hyperlink ref="C317" r:id="rId310" xr:uid="{DD66AAF5-1F82-4989-83DD-679F1B1207BD}"/>
+    <hyperlink ref="C318" r:id="rId311" xr:uid="{641FFE53-A63C-4366-9137-728A2DB43118}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId311"/>
+  <pageSetup orientation="portrait" r:id="rId312"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: find articulation point
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FCE211C-C556-48BE-BC8F-B65FEE2C3AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF8B54ED-F680-4316-A0B7-75F7523F8B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="640">
   <si>
     <t>date</t>
   </si>
@@ -1934,6 +1934,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/critical-connections-in-a-network/</t>
+  </si>
+  <si>
+    <t>articulation point</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/articulation-point2616/1</t>
   </si>
 </sst>
 </file>
@@ -2204,7 +2210,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D319"/>
+  <dimension ref="A1:D320"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5712,6 +5718,17 @@
       </c>
       <c r="C319" s="4" t="s">
         <v>637</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A320" s="1">
+        <v>46324</v>
+      </c>
+      <c r="B320" t="s">
+        <v>638</v>
+      </c>
+      <c r="C320" s="4" t="s">
+        <v>639</v>
       </c>
     </row>
   </sheetData>
@@ -6028,8 +6045,9 @@
     <hyperlink ref="C317" r:id="rId310" xr:uid="{DD66AAF5-1F82-4989-83DD-679F1B1207BD}"/>
     <hyperlink ref="C318" r:id="rId311" xr:uid="{641FFE53-A63C-4366-9137-728A2DB43118}"/>
     <hyperlink ref="C319" r:id="rId312" xr:uid="{4CEDE5A8-A4B0-44B2-8114-3AAE69B1ED73}"/>
+    <hyperlink ref="C320" r:id="rId313" xr:uid="{86881DC1-1A22-4FE7-BF5E-CE0A0D7FADD4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId313"/>
+  <pageSetup orientation="portrait" r:id="rId314"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: shortest path with at most k consecutive identical characters
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF8B54ED-F680-4316-A0B7-75F7523F8B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2E96C1E-B238-4E51-9ABB-6788FA952069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="640">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="642">
   <si>
     <t>date</t>
   </si>
@@ -1940,6 +1940,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/articulation-point2616/1</t>
+  </si>
+  <si>
+    <t>shortest path with at most k consecutive identical characters</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/shortest-path-with-at-most-k-consecutive-identical-characters/</t>
   </si>
 </sst>
 </file>
@@ -2210,7 +2216,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D320"/>
+  <dimension ref="A1:D321"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5729,6 +5735,17 @@
       </c>
       <c r="C320" s="4" t="s">
         <v>639</v>
+      </c>
+    </row>
+    <row r="321" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A321" s="1">
+        <v>46325</v>
+      </c>
+      <c r="B321" t="s">
+        <v>640</v>
+      </c>
+      <c r="C321" s="4" t="s">
+        <v>641</v>
       </c>
     </row>
   </sheetData>
@@ -6046,8 +6063,9 @@
     <hyperlink ref="C318" r:id="rId311" xr:uid="{641FFE53-A63C-4366-9137-728A2DB43118}"/>
     <hyperlink ref="C319" r:id="rId312" xr:uid="{4CEDE5A8-A4B0-44B2-8114-3AAE69B1ED73}"/>
     <hyperlink ref="C320" r:id="rId313" xr:uid="{86881DC1-1A22-4FE7-BF5E-CE0A0D7FADD4}"/>
+    <hyperlink ref="C321" r:id="rId314" xr:uid="{34A025CF-40AC-41F7-810B-06BF59D2FE07}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId314"/>
+  <pageSetup orientation="portrait" r:id="rId315"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Probem: twisted mirror path count
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2E96C1E-B238-4E51-9ABB-6788FA952069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF068BA-B5CD-41D0-8A0E-79A25450BC8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="642">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="644">
   <si>
     <t>date</t>
   </si>
@@ -1946,6 +1946,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/shortest-path-with-at-most-k-consecutive-identical-characters/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/twisted-mirror-path-count/</t>
+  </si>
+  <si>
+    <t>twisted mirror path count</t>
   </si>
 </sst>
 </file>
@@ -2216,7 +2222,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D321"/>
+  <dimension ref="A1:D322"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -5746,6 +5752,17 @@
       </c>
       <c r="C321" s="4" t="s">
         <v>641</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A322" s="1">
+        <v>46326</v>
+      </c>
+      <c r="B322" t="s">
+        <v>643</v>
+      </c>
+      <c r="C322" s="4" t="s">
+        <v>642</v>
       </c>
     </row>
   </sheetData>
@@ -6064,8 +6081,9 @@
     <hyperlink ref="C319" r:id="rId312" xr:uid="{4CEDE5A8-A4B0-44B2-8114-3AAE69B1ED73}"/>
     <hyperlink ref="C320" r:id="rId313" xr:uid="{86881DC1-1A22-4FE7-BF5E-CE0A0D7FADD4}"/>
     <hyperlink ref="C321" r:id="rId314" xr:uid="{34A025CF-40AC-41F7-810B-06BF59D2FE07}"/>
+    <hyperlink ref="C322" r:id="rId315" xr:uid="{C095830A-769F-4C71-BD9C-1139F4647623}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId315"/>
+  <pageSetup orientation="portrait" r:id="rId316"/>
 </worksheet>
 </file>
</xml_diff>